<commit_message>
Primer avance: unificación y categorización de datos 2017-2025
</commit_message>
<xml_diff>
--- a/Resultados de la votación 2017.xlsx
+++ b/Resultados de la votación 2017.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5fa8a9efe53b17c/Documentos/TP FINAL DATOS/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_936B57F7DC346A8067A2C4370A63FFA92E0F8519" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="465" windowWidth="28275" windowHeight="12240"/>
+    <workbookView minimized="1" xWindow="2520" yWindow="1836" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -15,7 +21,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$137</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$42:$G$65</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -493,10 +512,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -771,7 +790,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -784,7 +803,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -793,100 +812,100 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -895,7 +914,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -904,25 +923,25 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -931,28 +950,28 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -971,14 +990,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1016,7 +1038,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1088,7 +1110,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1261,25 +1283,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H146"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="51.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" style="4" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="9.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="51.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="16.88671875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.44140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="5" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="5" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>118</v>
       </c>
@@ -1302,7 +1324,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9">
         <v>959</v>
       </c>
@@ -1323,7 +1345,7 @@
       </c>
       <c r="G2" s="13"/>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="14">
         <v>506</v>
       </c>
@@ -1344,7 +1366,7 @@
       </c>
       <c r="G3" s="17"/>
     </row>
-    <row r="4" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14">
         <v>487</v>
       </c>
@@ -1365,7 +1387,7 @@
       </c>
       <c r="G4" s="17"/>
     </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="14">
         <v>482</v>
       </c>
@@ -1386,7 +1408,7 @@
       </c>
       <c r="G5" s="17"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="14">
         <v>446</v>
       </c>
@@ -1407,7 +1429,7 @@
       </c>
       <c r="G6" s="17"/>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>393</v>
       </c>
@@ -1428,7 +1450,7 @@
       </c>
       <c r="G7" s="17"/>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>373</v>
       </c>
@@ -1449,7 +1471,7 @@
       </c>
       <c r="G8" s="17"/>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>325</v>
       </c>
@@ -1470,7 +1492,7 @@
       </c>
       <c r="G9" s="17"/>
     </row>
-    <row r="10" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>280</v>
       </c>
@@ -1491,7 +1513,7 @@
       </c>
       <c r="G10" s="17"/>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>220</v>
       </c>
@@ -1512,7 +1534,7 @@
       </c>
       <c r="G11" s="17"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>191</v>
       </c>
@@ -1533,7 +1555,7 @@
       </c>
       <c r="G12" s="17"/>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>177</v>
       </c>
@@ -1554,7 +1576,7 @@
       </c>
       <c r="G13" s="17"/>
     </row>
-    <row r="14" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
         <v>146</v>
       </c>
@@ -1575,7 +1597,7 @@
       </c>
       <c r="G14" s="17"/>
     </row>
-    <row r="15" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>115</v>
       </c>
@@ -1596,7 +1618,7 @@
       </c>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
         <v>89</v>
       </c>
@@ -1620,7 +1642,7 @@
         <v>7190962</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="25">
         <v>84</v>
       </c>
@@ -1643,7 +1665,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="25">
         <v>81</v>
       </c>
@@ -1666,7 +1688,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="25">
         <v>72</v>
       </c>
@@ -1689,7 +1711,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="25">
         <v>67</v>
       </c>
@@ -1712,7 +1734,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="30">
         <v>55</v>
       </c>
@@ -1735,7 +1757,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
         <v>984</v>
       </c>
@@ -1756,7 +1778,7 @@
       </c>
       <c r="G22" s="13"/>
     </row>
-    <row r="23" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="25">
         <v>962</v>
       </c>
@@ -1779,7 +1801,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="14">
         <v>920</v>
       </c>
@@ -1800,7 +1822,7 @@
       </c>
       <c r="G24" s="17"/>
     </row>
-    <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="14">
         <v>800</v>
       </c>
@@ -1821,7 +1843,7 @@
       </c>
       <c r="G25" s="17"/>
     </row>
-    <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="14">
         <v>768</v>
       </c>
@@ -1842,7 +1864,7 @@
       </c>
       <c r="G26" s="17"/>
     </row>
-    <row r="27" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="14">
         <v>569</v>
       </c>
@@ -1863,7 +1885,7 @@
       </c>
       <c r="G27" s="17"/>
     </row>
-    <row r="28" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="25">
         <v>553</v>
       </c>
@@ -1886,7 +1908,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="25">
         <v>256</v>
       </c>
@@ -1909,7 +1931,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="25">
         <v>250</v>
       </c>
@@ -1932,7 +1954,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="14">
         <v>225</v>
       </c>
@@ -1953,7 +1975,7 @@
       </c>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="25">
         <v>206</v>
       </c>
@@ -1976,7 +1998,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="25">
         <v>197</v>
       </c>
@@ -1999,7 +2021,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="25">
         <v>196</v>
       </c>
@@ -2022,7 +2044,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="25">
         <v>188</v>
       </c>
@@ -2045,7 +2067,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="25">
         <v>172</v>
       </c>
@@ -2068,7 +2090,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="14">
         <v>170</v>
       </c>
@@ -2092,7 +2114,7 @@
         <v>7140125</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="25">
         <v>148</v>
       </c>
@@ -2115,7 +2137,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A39" s="25">
         <v>136</v>
       </c>
@@ -2138,7 +2160,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="25">
         <v>95</v>
       </c>
@@ -2161,7 +2183,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="34.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="30">
         <v>48</v>
       </c>
@@ -2184,7 +2206,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9">
         <v>763</v>
       </c>
@@ -2205,7 +2227,7 @@
       </c>
       <c r="G42" s="13"/>
     </row>
-    <row r="43" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="14">
         <v>573</v>
       </c>
@@ -2226,7 +2248,7 @@
       </c>
       <c r="G43" s="20"/>
     </row>
-    <row r="44" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="14">
         <v>528</v>
       </c>
@@ -2247,7 +2269,7 @@
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="14">
         <v>471</v>
       </c>
@@ -2268,7 +2290,7 @@
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="14">
         <v>435</v>
       </c>
@@ -2289,7 +2311,7 @@
       </c>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A47" s="14">
         <v>416</v>
       </c>
@@ -2310,7 +2332,7 @@
       </c>
       <c r="G47" s="20"/>
     </row>
-    <row r="48" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A48" s="14">
         <v>373</v>
       </c>
@@ -2331,7 +2353,7 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49" s="25">
         <v>354</v>
       </c>
@@ -2354,7 +2376,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="14">
         <v>324</v>
       </c>
@@ -2375,7 +2397,7 @@
       </c>
       <c r="G50" s="17"/>
     </row>
-    <row r="51" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="25">
         <v>268</v>
       </c>
@@ -2398,7 +2420,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="25">
         <v>227</v>
       </c>
@@ -2421,7 +2443,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A53" s="25">
         <v>225</v>
       </c>
@@ -2444,7 +2466,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="25">
         <v>192</v>
       </c>
@@ -2467,7 +2489,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="14">
         <v>191</v>
       </c>
@@ -2491,7 +2513,7 @@
         <v>8503370</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="25">
         <v>135</v>
       </c>
@@ -2514,7 +2536,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="25">
         <v>131</v>
       </c>
@@ -2537,7 +2559,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" s="25">
         <v>118</v>
       </c>
@@ -2560,7 +2582,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A59" s="25">
         <v>100</v>
       </c>
@@ -2583,7 +2605,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="25">
         <v>95</v>
       </c>
@@ -2606,7 +2628,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A61" s="25">
         <v>91</v>
       </c>
@@ -2629,7 +2651,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="25">
         <v>70</v>
       </c>
@@ -2652,7 +2674,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A63" s="25">
         <v>63</v>
       </c>
@@ -2675,7 +2697,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="25">
         <v>43</v>
       </c>
@@ -2698,7 +2720,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="30">
         <v>41</v>
       </c>
@@ -2721,7 +2743,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="9">
         <v>800</v>
       </c>
@@ -2742,7 +2764,7 @@
       </c>
       <c r="G66" s="13"/>
     </row>
-    <row r="67" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A67" s="14">
         <v>788</v>
       </c>
@@ -2763,7 +2785,7 @@
       </c>
       <c r="G67" s="17"/>
     </row>
-    <row r="68" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="14">
         <v>597</v>
       </c>
@@ -2784,7 +2806,7 @@
       </c>
       <c r="G68" s="17"/>
     </row>
-    <row r="69" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A69" s="14">
         <v>489</v>
       </c>
@@ -2805,7 +2827,7 @@
       </c>
       <c r="G69" s="17"/>
     </row>
-    <row r="70" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A70" s="14">
         <v>238</v>
       </c>
@@ -2826,7 +2848,7 @@
       </c>
       <c r="G70" s="17"/>
     </row>
-    <row r="71" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="14">
         <v>217</v>
       </c>
@@ -2847,7 +2869,7 @@
       </c>
       <c r="G71" s="17"/>
     </row>
-    <row r="72" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A72" s="14">
         <v>209</v>
       </c>
@@ -2868,7 +2890,7 @@
       </c>
       <c r="G72" s="17"/>
     </row>
-    <row r="73" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="14">
         <v>98</v>
       </c>
@@ -2892,7 +2914,7 @@
         <v>5967442</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A74" s="30">
         <v>97</v>
       </c>
@@ -2915,7 +2937,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="39">
         <v>805</v>
       </c>
@@ -2936,7 +2958,7 @@
       </c>
       <c r="G75" s="41"/>
     </row>
-    <row r="76" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A76" s="42">
         <v>743</v>
       </c>
@@ -2959,7 +2981,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="77" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A77" s="48">
         <v>555</v>
       </c>
@@ -2980,7 +3002,7 @@
       </c>
       <c r="G77" s="49"/>
     </row>
-    <row r="78" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A78" s="48">
         <v>369</v>
       </c>
@@ -3001,7 +3023,7 @@
       </c>
       <c r="G78" s="49"/>
     </row>
-    <row r="79" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A79" s="48">
         <v>267</v>
       </c>
@@ -3022,7 +3044,7 @@
       </c>
       <c r="G79" s="50"/>
     </row>
-    <row r="80" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A80" s="48">
         <v>254</v>
       </c>
@@ -3043,7 +3065,7 @@
       </c>
       <c r="G80" s="50"/>
     </row>
-    <row r="81" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A81" s="48">
         <v>249</v>
       </c>
@@ -3064,7 +3086,7 @@
       </c>
       <c r="G81" s="49"/>
     </row>
-    <row r="82" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A82" s="51">
         <v>185</v>
       </c>
@@ -3087,7 +3109,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="83" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A83" s="48">
         <v>111</v>
       </c>
@@ -3111,7 +3133,7 @@
         <v>5527155</v>
       </c>
     </row>
-    <row r="84" spans="1:7" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A84" s="52">
         <v>12</v>
       </c>
@@ -3134,7 +3156,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="9">
         <v>1717</v>
       </c>
@@ -3155,7 +3177,7 @@
       </c>
       <c r="G85" s="13"/>
     </row>
-    <row r="86" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="54">
         <v>1360</v>
       </c>
@@ -3176,7 +3198,7 @@
       </c>
       <c r="G86" s="17"/>
     </row>
-    <row r="87" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="14">
         <v>1193</v>
       </c>
@@ -3197,7 +3219,7 @@
       </c>
       <c r="G87" s="17"/>
     </row>
-    <row r="88" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88" s="14">
         <v>923</v>
       </c>
@@ -3218,7 +3240,7 @@
       </c>
       <c r="G88" s="17"/>
     </row>
-    <row r="89" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89" s="14">
         <v>847</v>
       </c>
@@ -3239,7 +3261,7 @@
       </c>
       <c r="G89" s="17"/>
     </row>
-    <row r="90" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A90" s="25">
         <v>785</v>
       </c>
@@ -3262,7 +3284,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="91" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A91" s="14">
         <v>757</v>
       </c>
@@ -3283,7 +3305,7 @@
       </c>
       <c r="G91" s="20"/>
     </row>
-    <row r="92" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="14">
         <v>494</v>
       </c>
@@ -3307,7 +3329,7 @@
         <v>8375854</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A93" s="25">
         <v>344</v>
       </c>
@@ -3330,7 +3352,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A94" s="25">
         <v>298</v>
       </c>
@@ -3353,7 +3375,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A95" s="25">
         <v>245</v>
       </c>
@@ -3376,7 +3398,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A96" s="25">
         <v>202</v>
       </c>
@@ -3399,7 +3421,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="25">
         <v>202</v>
       </c>
@@ -3422,7 +3444,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A98" s="25">
         <v>200</v>
       </c>
@@ -3445,7 +3467,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="25">
         <v>192</v>
       </c>
@@ -3468,7 +3490,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="25">
         <v>161</v>
       </c>
@@ -3491,7 +3513,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:7" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30">
         <v>97</v>
       </c>
@@ -3514,7 +3536,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="9">
         <v>542</v>
       </c>
@@ -3535,7 +3557,7 @@
       </c>
       <c r="G102" s="13"/>
     </row>
-    <row r="103" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A103" s="14">
         <v>339</v>
       </c>
@@ -3556,7 +3578,7 @@
       </c>
       <c r="G103" s="17"/>
     </row>
-    <row r="104" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A104" s="14">
         <v>187</v>
       </c>
@@ -3577,7 +3599,7 @@
       </c>
       <c r="G104" s="17"/>
     </row>
-    <row r="105" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A105" s="14">
         <v>182</v>
       </c>
@@ -3598,7 +3620,7 @@
       </c>
       <c r="G105" s="17"/>
     </row>
-    <row r="106" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A106" s="14">
         <v>114</v>
       </c>
@@ -3622,7 +3644,7 @@
         <v>5966912</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="25">
         <v>63</v>
       </c>
@@ -3645,7 +3667,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="108" spans="1:7" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:7" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A108" s="30">
         <v>60</v>
       </c>
@@ -3668,7 +3690,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A109" s="9">
         <v>2832</v>
       </c>
@@ -3689,7 +3711,7 @@
       </c>
       <c r="G109" s="13"/>
     </row>
-    <row r="110" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A110" s="14">
         <v>1468</v>
       </c>
@@ -3710,7 +3732,7 @@
       </c>
       <c r="G110" s="17"/>
     </row>
-    <row r="111" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A111" s="14">
         <v>1222</v>
       </c>
@@ -3731,7 +3753,7 @@
       </c>
       <c r="G111" s="17"/>
     </row>
-    <row r="112" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A112" s="14">
         <v>1130</v>
       </c>
@@ -3752,7 +3774,7 @@
       </c>
       <c r="G112" s="17"/>
     </row>
-    <row r="113" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="14">
         <v>1033</v>
       </c>
@@ -3773,7 +3795,7 @@
       </c>
       <c r="G113" s="17"/>
     </row>
-    <row r="114" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="14">
         <v>940</v>
       </c>
@@ -3794,7 +3816,7 @@
       </c>
       <c r="G114" s="17"/>
     </row>
-    <row r="115" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A115" s="14">
         <v>915</v>
       </c>
@@ -3815,7 +3837,7 @@
       </c>
       <c r="G115" s="17"/>
     </row>
-    <row r="116" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A116" s="25">
         <v>859</v>
       </c>
@@ -3838,7 +3860,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A117" s="25">
         <v>855</v>
       </c>
@@ -3861,7 +3883,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A118" s="25">
         <v>811</v>
       </c>
@@ -3884,7 +3906,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="14">
         <v>742</v>
       </c>
@@ -3905,7 +3927,7 @@
       </c>
       <c r="G119" s="17"/>
     </row>
-    <row r="120" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="25">
         <v>571</v>
       </c>
@@ -3928,7 +3950,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="25">
         <v>535</v>
       </c>
@@ -3951,7 +3973,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="14">
         <v>495</v>
       </c>
@@ -3972,7 +3994,7 @@
       </c>
       <c r="G122" s="17"/>
     </row>
-    <row r="123" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A123" s="25">
         <v>392</v>
       </c>
@@ -3995,7 +4017,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="43">
         <v>388</v>
       </c>
@@ -4018,7 +4040,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="125" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A125" s="25">
         <v>379</v>
       </c>
@@ -4041,7 +4063,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="126" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="25">
         <v>298</v>
       </c>
@@ -4064,7 +4086,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="25">
         <v>286</v>
       </c>
@@ -4087,7 +4109,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A128" s="25">
         <v>280</v>
       </c>
@@ -4110,7 +4132,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="129" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A129" s="14">
         <v>272</v>
       </c>
@@ -4134,7 +4156,7 @@
         <v>8453500</v>
       </c>
     </row>
-    <row r="130" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="25">
         <v>207</v>
       </c>
@@ -4157,7 +4179,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="131" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="25">
         <v>204</v>
       </c>
@@ -4180,7 +4202,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A132" s="25">
         <v>191</v>
       </c>
@@ -4203,7 +4225,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A133" s="25">
         <v>183</v>
       </c>
@@ -4226,7 +4248,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A134" s="25">
         <v>167</v>
       </c>
@@ -4249,7 +4271,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="135" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A135" s="25">
         <v>154</v>
       </c>
@@ -4272,7 +4294,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="136" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="25">
         <v>133</v>
       </c>
@@ -4296,7 +4318,7 @@
       </c>
       <c r="H136" s="8"/>
     </row>
-    <row r="137" spans="1:8" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A137" s="25">
         <v>56</v>
       </c>
@@ -4319,7 +4341,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A138" s="56">
         <v>1274</v>
       </c>
@@ -4340,7 +4362,7 @@
       </c>
       <c r="G138" s="57"/>
     </row>
-    <row r="139" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="48">
         <v>995</v>
       </c>
@@ -4361,7 +4383,7 @@
       </c>
       <c r="G139" s="49"/>
     </row>
-    <row r="140" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A140" s="48">
         <v>887</v>
       </c>
@@ -4382,7 +4404,7 @@
       </c>
       <c r="G140" s="49"/>
     </row>
-    <row r="141" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A141" s="48">
         <v>580</v>
       </c>
@@ -4403,7 +4425,7 @@
       </c>
       <c r="G141" s="49"/>
     </row>
-    <row r="142" spans="1:8" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A142" s="51">
         <v>553</v>
       </c>
@@ -4426,7 +4448,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="143" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A143" s="51">
         <v>360</v>
       </c>
@@ -4449,7 +4471,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="144" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A144" s="51">
         <v>263</v>
       </c>
@@ -4472,7 +4494,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="145" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A145" s="48">
         <v>218</v>
       </c>
@@ -4493,7 +4515,7 @@
       </c>
       <c r="G145" s="49"/>
     </row>
-    <row r="146" spans="1:7" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:7" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A146" s="58">
         <v>208</v>
       </c>
@@ -4518,7 +4540,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A79:L88">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A79:L88">
     <sortCondition descending="1" ref="A79:A88"/>
   </sortState>
   <pageMargins left="0.23622047244094491" right="0.15748031496062992" top="0.47244094488188981" bottom="0.31496062992125984" header="0.19685039370078741" footer="0.31496062992125984"/>
@@ -4530,18 +4552,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>